<commit_message>
AO Lapeyre : motorisés à 100 €, total 5 240 € HT/an
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QNKU3vJ4q3pKM5CqtQ7baF
</commit_message>
<xml_diff>
--- a/Lapeyre_Positionnement_Chiffrage_RhoneAlpes.xlsx
+++ b/Lapeyre_Positionnement_Chiffrage_RhoneAlpes.xlsx
@@ -3784,10 +3784,10 @@
         <v>2</v>
       </c>
       <c r="E5" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F5" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6">
@@ -3875,7 +3875,7 @@
       <c r="D9" s="15" t="inlineStr"/>
       <c r="E9" s="15" t="inlineStr"/>
       <c r="F9" s="15" t="n">
-        <v>540</v>
+        <v>560</v>
       </c>
     </row>
     <row r="10">
@@ -3984,10 +3984,10 @@
         <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F14" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15">
@@ -4008,10 +4008,10 @@
         <v>2</v>
       </c>
       <c r="E15" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F15" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16">
@@ -4056,10 +4056,10 @@
         <v>2</v>
       </c>
       <c r="E17" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F17" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18">
@@ -4075,7 +4075,7 @@
       <c r="D18" s="15" t="inlineStr"/>
       <c r="E18" s="15" t="inlineStr"/>
       <c r="F18" s="15" t="n">
-        <v>540</v>
+        <v>600</v>
       </c>
     </row>
     <row r="19">
@@ -4096,10 +4096,10 @@
         <v>2</v>
       </c>
       <c r="E19" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F19" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20">
@@ -4187,7 +4187,7 @@
       <c r="D23" s="15" t="inlineStr"/>
       <c r="E23" s="15" t="inlineStr"/>
       <c r="F23" s="15" t="n">
-        <v>380</v>
+        <v>400</v>
       </c>
     </row>
     <row r="24">
@@ -4416,10 +4416,10 @@
         <v>2</v>
       </c>
       <c r="E33" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F33" t="n">
-        <v>160</v>
+        <v>200</v>
       </c>
     </row>
     <row r="34">
@@ -4435,7 +4435,7 @@
       <c r="D34" s="15" t="inlineStr"/>
       <c r="E34" s="15" t="inlineStr"/>
       <c r="F34" s="15" t="n">
-        <v>960</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="35">
@@ -4688,7 +4688,7 @@
         <v>70</v>
       </c>
       <c r="F46" t="n">
-        <v>5100</v>
+        <v>5240</v>
       </c>
     </row>
     <row r="47">
@@ -4698,9 +4698,10 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>4590</v>
-      </c>
-    </row>
+        <v>4716</v>
+      </c>
+    </row>
+    <row r="48"/>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>

</xml_diff>